<commit_message>
Revise wording in 3-2
</commit_message>
<xml_diff>
--- a/docs/handouts/chapter_3_2_handout.xlsx
+++ b/docs/handouts/chapter_3_2_handout.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\RData\BYUI-Timeseries-Drafts\handouts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\craigaj\Documents\GitHub\timeseries\handouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3188E1FC-9749-4475-91A3-388780982B23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C604117F-4FD3-42F2-99D7-3C91E8B02DD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CB73943A-C465-40BE-817C-B9991112161C}"/>
+    <workbookView xWindow="-11055" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{CB73943A-C465-40BE-817C-B9991112161C}"/>
   </bookViews>
   <sheets>
     <sheet name="Workbook" sheetId="2" r:id="rId1"/>
@@ -81,7 +81,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -94,8 +94,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -113,33 +119,45 @@
       <top style="thin">
         <color theme="1"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
-        <color theme="1"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FFB3B3B3"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
       <bottom style="thin">
         <color theme="1"/>
       </bottom>
@@ -149,46 +167,7 @@
       <left/>
       <right/>
       <top style="medium">
-        <color rgb="FFB3B3B3"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFB3B3B3"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
         <color theme="1"/>
@@ -200,9 +179,99 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="medium">
-        <color rgb="FFB3B3B3"/>
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -210,37 +279,52 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -369,10 +453,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -581,8 +662,8 @@
       <xdr:rowOff>60833</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="202298" cy="221214"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="10" name="TextBox 9">
@@ -627,10 +708,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -664,7 +742,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="10" name="TextBox 9">
@@ -729,8 +807,8 @@
       <xdr:rowOff>60833</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="186077" cy="221214"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="17" name="TextBox 16">
@@ -775,10 +853,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -812,7 +887,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="17" name="TextBox 16">
@@ -918,7 +993,6 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr/>
           <a:endParaRPr lang="en-US" sz="1200"/>
         </a:p>
       </xdr:txBody>
@@ -933,8 +1007,8 @@
       <xdr:rowOff>60833</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="202298" cy="221214"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="13" name="TextBox 12">
@@ -979,10 +1053,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -1016,7 +1087,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="13" name="TextBox 12">
@@ -1081,8 +1152,8 @@
       <xdr:rowOff>53213</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="186077" cy="221214"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="21" name="TextBox 20">
@@ -1127,10 +1198,7 @@
               <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMath>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -1164,7 +1232,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="21" name="TextBox 20">
@@ -1542,134 +1610,134 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ABFF2E6-1E13-48EF-9BE3-D6C90C46BEC8}">
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.88671875" customWidth="1"/>
+    <col min="1" max="1" width="11.90625" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.88671875" customWidth="1"/>
-    <col min="10" max="10" width="9.6640625" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.90625" customWidth="1"/>
+    <col min="10" max="10" width="9.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:5" ht="48.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
       <c r="D1" s="9"/>
     </row>
-    <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A2" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="2"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="5"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="1"/>
     </row>
-    <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="11">
         <v>1</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="5">
         <v>4.4000000000000004</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="11"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="12"/>
     </row>
-    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="11">
         <v>2</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="5">
         <v>4.2</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="11"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="12"/>
     </row>
-    <row r="5" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="11">
         <v>3</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="5">
         <v>4.2</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="11"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="12"/>
     </row>
-    <row r="6" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="11">
         <v>4</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="5">
         <v>4</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="11"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="12"/>
     </row>
-    <row r="7" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="11">
         <v>5</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="5">
         <v>4.4000000000000004</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="11"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="12"/>
     </row>
-    <row r="8" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="11">
         <v>6</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="5">
         <v>4.7</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="11"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="12"/>
     </row>
-    <row r="9" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="11">
         <v>7</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="5">
         <v>4.9000000000000004</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="11"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="12"/>
     </row>
-    <row r="10" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="11">
         <v>8</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="5">
         <v>5.3</v>
       </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="11"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="12"/>
     </row>
-    <row r="11" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="11">
         <v>9</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="5">
         <v>5.4</v>
       </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="11"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="12"/>
     </row>
-    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="4">
+    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="13">
         <v>10</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="14">
         <v>5.5</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="8"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1682,6 +1750,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010070F75838E79B0E48B83E8E3F5479A3A2" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2b0c304636f8f537543cd13f583db9d4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xmlns:ns4="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f089f22c5ce4e61126931f7622145b2" ns3:_="" ns4:_="">
     <xsd:import namespace="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
@@ -1876,14 +1952,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1894,6 +1962,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5E1B631-90B0-4D19-A35E-F8DC8BE167A4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBDDC771-C014-4A48-9FCA-802C556EA1D0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1912,23 +1997,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5E1B631-90B0-4D19-A35E-F8DC8BE167A4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
   <ds:schemaRefs>

</xml_diff>